<commit_message>
feat(cuestionario): complementar flujo de cuestionario escenario 2
Implementa las validaciones y campos adicionales requeridos para completar el segundo escenario del flujo de cuestionario.
Asegura la integración con los selectores del proyecto AutomatizacionAF y optimiza los tiempos de espera entre transiciones.
</commit_message>
<xml_diff>
--- a/src/datos/SuitePruebas.xlsx
+++ b/src/datos/SuitePruebas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\AutomatizacionAF\src\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automatización\Git\AutomatizacionAF\src\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A155A4FD-CB18-4AB7-A46C-1480329278F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3E2163-F863-4752-A213-E0BB383AFBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-156" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CotizadorAF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1422" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="122">
   <si>
     <t>EscenarioPrueba</t>
   </si>
@@ -401,6 +401,9 @@
   </si>
   <si>
     <t>Cotizacion Optima Plus Mensual</t>
+  </si>
+  <si>
+    <t>$2,000.00 / $4,000.00 USD</t>
   </si>
 </sst>
 </file>
@@ -470,7 +473,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -480,7 +483,6 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1084,7 +1086,7 @@
       </c>
     </row>
     <row r="2" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" t="s">
         <v>103</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1187,7 +1189,7 @@
         <v>6</v>
       </c>
       <c r="AI2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK2" s="4"/>
       <c r="AM2" s="3"/>
@@ -1240,7 +1242,7 @@
       </c>
     </row>
     <row r="3" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" t="s">
         <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1271,7 +1273,7 @@
         <v>102</v>
       </c>
       <c r="K3" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="L3" t="s">
         <v>4</v>
@@ -1343,7 +1345,7 @@
         <v>6</v>
       </c>
       <c r="AI3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK3" s="4"/>
       <c r="AM3" s="3"/>
@@ -1396,7 +1398,7 @@
       </c>
     </row>
     <row r="4" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" t="s">
         <v>105</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1499,7 +1501,7 @@
         <v>6</v>
       </c>
       <c r="AI4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK4" s="4"/>
       <c r="AM4" s="3"/>
@@ -1552,7 +1554,7 @@
       </c>
     </row>
     <row r="5" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" t="s">
         <v>106</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1655,11 +1657,11 @@
         <v>6</v>
       </c>
       <c r="AI5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" t="s">
         <v>107</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1762,7 +1764,7 @@
         <v>6</v>
       </c>
       <c r="AI6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK6" s="4"/>
       <c r="AM6" s="3"/>
@@ -1815,7 +1817,7 @@
       </c>
     </row>
     <row r="7" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" t="s">
         <v>108</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1846,7 +1848,7 @@
         <v>111</v>
       </c>
       <c r="K7" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="L7" t="s">
         <v>4</v>
@@ -1918,7 +1920,7 @@
         <v>6</v>
       </c>
       <c r="AI7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK7" s="4"/>
       <c r="AM7" s="3"/>
@@ -1971,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" t="s">
         <v>109</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -2074,7 +2076,7 @@
         <v>6</v>
       </c>
       <c r="AI8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK8" s="4"/>
       <c r="AM8" s="3"/>
@@ -2127,7 +2129,7 @@
       </c>
     </row>
     <row r="9" spans="1:117" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" t="s">
         <v>110</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -2230,7 +2232,7 @@
         <v>6</v>
       </c>
       <c r="AI9" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:117" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat(113458):Cotización FAM ENG CODEX
Se realiza el flujo para la cotizacion Familiar en el idioma ingles
Respeta las reglas de negocio actualmente implementadas para el flujo en ESP.
</commit_message>
<xml_diff>
--- a/src/datos/SuitePruebas.xlsx
+++ b/src/datos/SuitePruebas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automatización\Git\AutomatizacionAF\src\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegobautistaluis/Git/AutomatizacionAF/src/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3E2163-F863-4752-A213-E0BB383AFBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE40AE5-7D73-164A-A5CC-C5351225B310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CotizadorAF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1422" uniqueCount="122">
   <si>
     <t>EscenarioPrueba</t>
   </si>
@@ -820,120 +820,120 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DM13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="50" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.5" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="23" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="23.42578125" customWidth="1"/>
-    <col min="28" max="28" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="23.5" customWidth="1"/>
+    <col min="28" max="28" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="25" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="26" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="14" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="27.28515625" customWidth="1"/>
-    <col min="60" max="60" width="17.28515625" customWidth="1"/>
-    <col min="61" max="61" width="21.140625" customWidth="1"/>
-    <col min="62" max="62" width="11.7109375" customWidth="1"/>
+    <col min="54" max="54" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="27.33203125" customWidth="1"/>
+    <col min="60" max="60" width="17.33203125" customWidth="1"/>
+    <col min="61" max="61" width="21.1640625" customWidth="1"/>
+    <col min="62" max="62" width="11.6640625" customWidth="1"/>
     <col min="63" max="63" width="17" customWidth="1"/>
-    <col min="65" max="65" width="11.7109375" customWidth="1"/>
-    <col min="66" max="66" width="16.140625" customWidth="1"/>
-    <col min="67" max="67" width="19.140625" customWidth="1"/>
-    <col min="68" max="68" width="22.7109375" customWidth="1"/>
-    <col min="69" max="69" width="20.7109375" customWidth="1"/>
-    <col min="70" max="70" width="13.28515625" customWidth="1"/>
+    <col min="65" max="65" width="11.6640625" customWidth="1"/>
+    <col min="66" max="66" width="16.1640625" customWidth="1"/>
+    <col min="67" max="67" width="19.1640625" customWidth="1"/>
+    <col min="68" max="68" width="22.6640625" customWidth="1"/>
+    <col min="69" max="69" width="20.6640625" customWidth="1"/>
+    <col min="70" max="70" width="13.33203125" customWidth="1"/>
     <col min="71" max="71" width="15" customWidth="1"/>
-    <col min="74" max="74" width="27.7109375" customWidth="1"/>
-    <col min="75" max="75" width="14.42578125" customWidth="1"/>
-    <col min="76" max="76" width="20.42578125" customWidth="1"/>
-    <col min="77" max="77" width="22.140625" customWidth="1"/>
-    <col min="78" max="78" width="26.7109375" customWidth="1"/>
-    <col min="79" max="79" width="28.85546875" customWidth="1"/>
-    <col min="80" max="80" width="13.7109375" customWidth="1"/>
-    <col min="81" max="81" width="22.85546875" customWidth="1"/>
-    <col min="82" max="82" width="20.7109375" customWidth="1"/>
-    <col min="83" max="83" width="23.28515625" customWidth="1"/>
-    <col min="84" max="84" width="31.140625" customWidth="1"/>
-    <col min="85" max="85" width="26.42578125" customWidth="1"/>
-    <col min="86" max="86" width="23.7109375" customWidth="1"/>
-    <col min="87" max="87" width="17.28515625" customWidth="1"/>
-    <col min="88" max="88" width="19.28515625" customWidth="1"/>
-    <col min="89" max="89" width="19.42578125" customWidth="1"/>
-    <col min="90" max="90" width="17.140625" customWidth="1"/>
-    <col min="91" max="91" width="17.7109375" customWidth="1"/>
-    <col min="92" max="92" width="14.7109375" customWidth="1"/>
-    <col min="93" max="93" width="26.7109375" customWidth="1"/>
-    <col min="94" max="94" width="27.42578125" customWidth="1"/>
-    <col min="95" max="95" width="17.140625" customWidth="1"/>
-    <col min="96" max="96" width="17.85546875" customWidth="1"/>
+    <col min="74" max="74" width="27.6640625" customWidth="1"/>
+    <col min="75" max="75" width="14.5" customWidth="1"/>
+    <col min="76" max="76" width="20.5" customWidth="1"/>
+    <col min="77" max="77" width="22.1640625" customWidth="1"/>
+    <col min="78" max="78" width="26.6640625" customWidth="1"/>
+    <col min="79" max="79" width="28.83203125" customWidth="1"/>
+    <col min="80" max="80" width="13.6640625" customWidth="1"/>
+    <col min="81" max="81" width="22.83203125" customWidth="1"/>
+    <col min="82" max="82" width="20.6640625" customWidth="1"/>
+    <col min="83" max="83" width="23.33203125" customWidth="1"/>
+    <col min="84" max="84" width="31.1640625" customWidth="1"/>
+    <col min="85" max="85" width="26.5" customWidth="1"/>
+    <col min="86" max="86" width="23.6640625" customWidth="1"/>
+    <col min="87" max="87" width="17.33203125" customWidth="1"/>
+    <col min="88" max="88" width="19.33203125" customWidth="1"/>
+    <col min="89" max="89" width="19.5" customWidth="1"/>
+    <col min="90" max="90" width="17.1640625" customWidth="1"/>
+    <col min="91" max="91" width="17.6640625" customWidth="1"/>
+    <col min="92" max="92" width="14.6640625" customWidth="1"/>
+    <col min="93" max="93" width="26.6640625" customWidth="1"/>
+    <col min="94" max="94" width="27.5" customWidth="1"/>
+    <col min="95" max="95" width="17.1640625" customWidth="1"/>
+    <col min="96" max="96" width="17.83203125" customWidth="1"/>
     <col min="97" max="97" width="19" customWidth="1"/>
     <col min="98" max="99" width="29" customWidth="1"/>
-    <col min="100" max="100" width="17.28515625" customWidth="1"/>
+    <col min="100" max="100" width="17.33203125" customWidth="1"/>
     <col min="101" max="101" width="20" customWidth="1"/>
-    <col min="102" max="102" width="17.7109375" customWidth="1"/>
-    <col min="103" max="107" width="20.5703125" customWidth="1"/>
+    <col min="102" max="102" width="17.6640625" customWidth="1"/>
+    <col min="103" max="107" width="20.5" customWidth="1"/>
     <col min="108" max="108" width="14" customWidth="1"/>
     <col min="109" max="109" width="15" customWidth="1"/>
-    <col min="110" max="110" width="19.28515625" customWidth="1"/>
-    <col min="111" max="111" width="13.85546875" customWidth="1"/>
-    <col min="112" max="112" width="21.7109375" customWidth="1"/>
+    <col min="110" max="110" width="19.33203125" customWidth="1"/>
+    <col min="111" max="111" width="13.83203125" customWidth="1"/>
+    <col min="112" max="112" width="21.6640625" customWidth="1"/>
     <col min="113" max="113" width="24" customWidth="1"/>
-    <col min="114" max="114" width="18.140625" customWidth="1"/>
-    <col min="115" max="115" width="21.28515625" customWidth="1"/>
-    <col min="116" max="116" width="22.5703125" customWidth="1"/>
-    <col min="117" max="117" width="14.85546875" customWidth="1"/>
+    <col min="114" max="114" width="18.1640625" customWidth="1"/>
+    <col min="115" max="115" width="21.33203125" customWidth="1"/>
+    <col min="116" max="116" width="22.5" customWidth="1"/>
+    <col min="117" max="117" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1085,9 +1085,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>26</v>
@@ -1111,13 +1111,13 @@
         <v>35</v>
       </c>
       <c r="I2" t="s">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="J2" t="s">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="K2" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="L2" t="s">
         <v>3</v>
@@ -1241,7 +1241,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>105</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>106</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>107</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>108</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>109</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:117" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>110</v>
       </c>
@@ -2235,20 +2235,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:117" x14ac:dyDescent="0.2">
       <c r="AU10" s="2"/>
       <c r="DM10" s="2"/>
     </row>
-    <row r="11" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:117" x14ac:dyDescent="0.2">
       <c r="G11" t="s">
         <v>42</v>
       </c>
       <c r="AU11" s="2"/>
     </row>
-    <row r="12" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:117" x14ac:dyDescent="0.2">
       <c r="BE12" s="1"/>
     </row>
-    <row r="13" spans="1:117" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:117" x14ac:dyDescent="0.2">
       <c r="E13" t="s">
         <v>24</v>
       </c>
@@ -2282,16 +2282,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91658F97-1B63-4028-A047-57A0079160D2}">
   <dimension ref="A1:AE4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="23.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="54.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="11.42578125" style="4"/>
+    <col min="1" max="2" width="23.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="54.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" style="4" customWidth="1"/>
+    <col min="6" max="16384" width="11.5" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="AE1" s="5"/>
     </row>
-    <row r="2" spans="1:31" ht="21.75" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:31" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>77</v>
       </c>
@@ -2327,10 +2327,10 @@
       </c>
       <c r="AE2" s="5"/>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
       <c r="AE3" s="5"/>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
       <c r="AE4" s="5"/>
     </row>
   </sheetData>
@@ -2345,12 +2345,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89217B83-F5AC-41B7-85ED-07DFA2DFDFF5}">
   <dimension ref="A1:BF24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="1" max="1" width="34.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>114</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>113</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>92</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>93</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>94</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>95</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>96</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>115</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>97</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>98</v>
       </c>
@@ -3812,7 +3812,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>99</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>100</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>117</v>
       </c>
@@ -4231,7 +4231,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
         <v>118</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>119</v>
       </c>
@@ -4543,7 +4543,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>120</v>
       </c>
@@ -4650,7 +4650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>103</v>
       </c>
@@ -4806,7 +4806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>104</v>
       </c>
@@ -4962,7 +4962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>105</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>106</v>
       </c>
@@ -5225,7 +5225,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>107</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>108</v>
       </c>
@@ -5537,7 +5537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>109</v>
       </c>
@@ -5693,7 +5693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>110</v>
       </c>

</xml_diff>